<commit_message>
gera de novo, corta dados da idade do pai para 50 anos para facilitar a comparacao com  tft feminina
</commit_message>
<xml_diff>
--- a/202505_resultados/ 2022 _TFT_por_UF.xlsx
+++ b/202505_resultados/ 2022 _TFT_por_UF.xlsx
@@ -381,7 +381,7 @@
         <v>1.769</v>
       </c>
       <c r="C2">
-        <v>1.777</v>
+        <v>1.762</v>
       </c>
     </row>
     <row r="3">
@@ -394,7 +394,7 @@
         <v>1.881</v>
       </c>
       <c r="C3">
-        <v>2.007</v>
+        <v>1.999</v>
       </c>
     </row>
     <row r="4">
@@ -407,7 +407,7 @@
         <v>1.995</v>
       </c>
       <c r="C4">
-        <v>2.072</v>
+        <v>2.054</v>
       </c>
     </row>
     <row r="5">
@@ -420,7 +420,7 @@
         <v>2.238</v>
       </c>
       <c r="C5">
-        <v>2.312</v>
+        <v>2.298</v>
       </c>
     </row>
     <row r="6">
@@ -433,7 +433,7 @@
         <v>1.726</v>
       </c>
       <c r="C6">
-        <v>1.788</v>
+        <v>1.774</v>
       </c>
     </row>
     <row r="7">
@@ -446,7 +446,7 @@
         <v>1.944</v>
       </c>
       <c r="C7">
-        <v>2.05</v>
+        <v>2.04</v>
       </c>
     </row>
     <row r="8">
@@ -459,7 +459,7 @@
         <v>1.779</v>
       </c>
       <c r="C8">
-        <v>1.803</v>
+        <v>1.786</v>
       </c>
     </row>
     <row r="9">
@@ -472,7 +472,7 @@
         <v>1.644</v>
       </c>
       <c r="C9">
-        <v>1.747</v>
+        <v>1.74</v>
       </c>
     </row>
     <row r="10">
@@ -485,7 +485,7 @@
         <v>1.579</v>
       </c>
       <c r="C10">
-        <v>1.627</v>
+        <v>1.623</v>
       </c>
     </row>
     <row r="11">
@@ -498,7 +498,7 @@
         <v>1.489</v>
       </c>
       <c r="C11">
-        <v>1.529</v>
+        <v>1.523</v>
       </c>
     </row>
     <row r="12">
@@ -511,7 +511,7 @@
         <v>1.465</v>
       </c>
       <c r="C12">
-        <v>1.48</v>
+        <v>1.471</v>
       </c>
     </row>
     <row r="13">
@@ -524,7 +524,7 @@
         <v>1.577</v>
       </c>
       <c r="C13">
-        <v>1.636</v>
+        <v>1.628</v>
       </c>
     </row>
     <row r="14">
@@ -537,7 +537,7 @@
         <v>1.548</v>
       </c>
       <c r="C14">
-        <v>1.61</v>
+        <v>1.604</v>
       </c>
     </row>
     <row r="15">
@@ -550,7 +550,7 @@
         <v>1.719</v>
       </c>
       <c r="C15">
-        <v>1.859</v>
+        <v>1.852</v>
       </c>
     </row>
     <row r="16">
@@ -563,7 +563,7 @@
         <v>1.516</v>
       </c>
       <c r="C16">
-        <v>1.617</v>
+        <v>1.606</v>
       </c>
     </row>
     <row r="17">
@@ -576,7 +576,7 @@
         <v>1.471</v>
       </c>
       <c r="C17">
-        <v>1.536</v>
+        <v>1.526</v>
       </c>
     </row>
     <row r="18">
@@ -589,7 +589,7 @@
         <v>1.463</v>
       </c>
       <c r="C18">
-        <v>1.453</v>
+        <v>1.439</v>
       </c>
     </row>
     <row r="19">
@@ -602,7 +602,7 @@
         <v>1.676</v>
       </c>
       <c r="C19">
-        <v>1.677</v>
+        <v>1.663</v>
       </c>
     </row>
     <row r="20">
@@ -615,7 +615,7 @@
         <v>1.39</v>
       </c>
       <c r="C20">
-        <v>1.433</v>
+        <v>1.417</v>
       </c>
     </row>
     <row r="21">
@@ -628,7 +628,7 @@
         <v>1.486</v>
       </c>
       <c r="C21">
-        <v>1.477</v>
+        <v>1.463</v>
       </c>
     </row>
     <row r="22">
@@ -641,7 +641,7 @@
         <v>1.587</v>
       </c>
       <c r="C22">
-        <v>1.594</v>
+        <v>1.573</v>
       </c>
     </row>
     <row r="23">
@@ -654,7 +654,7 @@
         <v>1.604</v>
       </c>
       <c r="C23">
-        <v>1.54</v>
+        <v>1.528</v>
       </c>
     </row>
     <row r="24">
@@ -667,7 +667,7 @@
         <v>1.484</v>
       </c>
       <c r="C24">
-        <v>1.481</v>
+        <v>1.46</v>
       </c>
     </row>
     <row r="25">
@@ -680,7 +680,7 @@
         <v>1.834</v>
       </c>
       <c r="C25">
-        <v>1.834</v>
+        <v>1.805</v>
       </c>
     </row>
     <row r="26">
@@ -693,7 +693,7 @@
         <v>1.946</v>
       </c>
       <c r="C26">
-        <v>1.89</v>
+        <v>1.88</v>
       </c>
     </row>
     <row r="27">
@@ -706,7 +706,7 @@
         <v>1.561</v>
       </c>
       <c r="C27">
-        <v>1.548</v>
+        <v>1.535</v>
       </c>
     </row>
     <row r="28">
@@ -719,7 +719,7 @@
         <v>1.471</v>
       </c>
       <c r="C28">
-        <v>1.542</v>
+        <v>1.519</v>
       </c>
     </row>
   </sheetData>

</xml_diff>